<commit_message>
more results + ensemble
</commit_message>
<xml_diff>
--- a/transformers/experiments/1d_vgg_vsu/summary.xlsx
+++ b/transformers/experiments/1d_vgg_vsu/summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,6 +570,176 @@
         <v>0.003538547138044306</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>batch_128</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>128</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9617510180337405</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9620418848167539</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.966695753344968</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9634962187318208</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.002774692267065034</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>lr_0.1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.6207097149505526</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.8801628853984875</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.8805991855730075</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.7938239286406825</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.1499214655265368</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>lr_0.01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>32</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9156486329261199</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.9354275741710296</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.9171029668411868</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9227263913127788</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.01102355687984476</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>lr_0.0001</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>32</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.9669866201279814</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9653868528214078</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.9684409540430483</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.9669381423308125</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.001527627618439875</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>wd_0.1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>32</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.6207097149505526</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.6207097149505526</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.6207097149505526</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.6207097149505526</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>